<commit_message>
Made some updates to the pacman
</commit_message>
<xml_diff>
--- a/Pacman humanECoG/10plusDelay.xlsx
+++ b/Pacman humanECoG/10plusDelay.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kokal\Desktop\Work\Github Repos\Mine\PacmanDelayedPrey\Pacman humanECoG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962E64AB-B555-4800-BDEA-9C956CE89859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{658F995E-9DA9-4961-A0CA-C69E7FAAE65F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="2265" windowWidth="21600" windowHeight="11295" xr2:uid="{53EA15CA-DBB7-6342-AD33-56E222683D56}"/>
+    <workbookView xWindow="2250" yWindow="2250" windowWidth="21600" windowHeight="11295" xr2:uid="{53EA15CA-DBB7-6342-AD33-56E222683D56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -54,12 +54,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -80,17 +86,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{9AA0E321-A595-4B3A-9F27-400214787B1D}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -445,429 +455,351 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>2</v>
-      </c>
-      <c r="B2">
+      <c r="A2" s="3">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>4</v>
+      <c r="C2" s="3">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>6</v>
       </c>
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3">
         <v>1</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="D3" s="3">
+        <v>6</v>
+      </c>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3">
         <v>1</v>
       </c>
-      <c r="D3">
+      <c r="C4" s="3">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3">
+        <v>8</v>
+      </c>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3">
+        <v>4</v>
+      </c>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="D6" s="3">
         <v>6</v>
       </c>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4">
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>2</v>
+      </c>
+      <c r="B7" s="3">
+        <v>3</v>
+      </c>
+      <c r="C7" s="3">
         <v>1</v>
       </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-      <c r="D4">
-        <v>8</v>
-      </c>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>4</v>
-      </c>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>2</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2</v>
-      </c>
-      <c r="B7">
-        <v>2</v>
-      </c>
-      <c r="C7">
-        <v>3</v>
-      </c>
-      <c r="D7">
+      <c r="D7" s="3">
         <v>8</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>2</v>
-      </c>
-      <c r="B8">
-        <v>3</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
+      <c r="A8" s="3">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3">
+        <v>2</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3">
         <v>4</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>2</v>
-      </c>
-      <c r="B9">
-        <v>3</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9">
+      <c r="A9" s="3">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3">
+        <v>2</v>
+      </c>
+      <c r="C9" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="D9" s="3">
         <v>6</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>2</v>
-      </c>
-      <c r="B10">
-        <v>3</v>
-      </c>
-      <c r="C10">
-        <v>3</v>
-      </c>
-      <c r="D10">
+      <c r="A10" s="3">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3">
+        <v>2</v>
+      </c>
+      <c r="C10" s="3">
+        <v>1</v>
+      </c>
+      <c r="D10" s="3">
         <v>8</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>3</v>
-      </c>
-      <c r="B11">
-        <v>2</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
+      <c r="A11" s="3">
+        <v>3</v>
+      </c>
+      <c r="B11" s="3">
+        <v>4</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0</v>
+      </c>
+      <c r="D11" s="3">
         <v>4</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>3</v>
-      </c>
-      <c r="B12">
-        <v>2</v>
-      </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-      <c r="D12">
+      <c r="A12" s="3">
+        <v>3</v>
+      </c>
+      <c r="B12" s="3">
+        <v>4</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="D12" s="3">
         <v>6</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>3</v>
-      </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-      <c r="C13">
-        <v>3</v>
-      </c>
-      <c r="D13">
+      <c r="A13" s="3">
+        <v>3</v>
+      </c>
+      <c r="B13" s="3">
+        <v>4</v>
+      </c>
+      <c r="C13" s="3">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3">
         <v>8</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>3</v>
-      </c>
-      <c r="B14">
-        <v>3</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
+      <c r="A14" s="3">
+        <v>4</v>
+      </c>
+      <c r="B14" s="3">
+        <v>3</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
         <v>4</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>3</v>
-      </c>
-      <c r="B15">
-        <v>3</v>
-      </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-      <c r="D15">
+      <c r="A15" s="3">
+        <v>4</v>
+      </c>
+      <c r="B15" s="3">
+        <v>3</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="D15" s="3">
         <v>6</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>3</v>
-      </c>
-      <c r="B16">
-        <v>3</v>
-      </c>
-      <c r="C16">
-        <v>3</v>
-      </c>
-      <c r="D16">
+      <c r="A16" s="3">
+        <v>4</v>
+      </c>
+      <c r="B16" s="3">
+        <v>3</v>
+      </c>
+      <c r="C16" s="3">
+        <v>1</v>
+      </c>
+      <c r="D16" s="3">
         <v>8</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>3</v>
-      </c>
-      <c r="B17">
-        <v>4</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
+      <c r="A17" s="3">
+        <v>4</v>
+      </c>
+      <c r="B17" s="3">
+        <v>5</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3">
         <v>4</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>3</v>
-      </c>
-      <c r="B18">
-        <v>4</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18">
+      <c r="A18" s="3">
+        <v>4</v>
+      </c>
+      <c r="B18" s="3">
+        <v>5</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="D18" s="3">
         <v>6</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>3</v>
-      </c>
-      <c r="B19">
-        <v>4</v>
-      </c>
-      <c r="C19">
-        <v>3</v>
-      </c>
-      <c r="D19">
+      <c r="A19" s="3">
+        <v>4</v>
+      </c>
+      <c r="B19" s="3">
+        <v>5</v>
+      </c>
+      <c r="C19" s="3">
+        <v>3</v>
+      </c>
+      <c r="D19" s="3">
         <v>8</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>4</v>
-      </c>
-      <c r="B20">
-        <v>3</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
+      <c r="A20" s="2">
+        <v>2</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2">
+        <v>0</v>
+      </c>
+      <c r="D20" s="3">
         <v>4</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>4</v>
-      </c>
-      <c r="B21">
-        <v>3</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-      <c r="D21">
-        <v>6</v>
+      <c r="A21" s="2">
+        <v>3</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3">
+        <v>4</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>4</v>
-      </c>
-      <c r="B22">
-        <v>3</v>
-      </c>
-      <c r="C22">
-        <v>3</v>
-      </c>
-      <c r="D22">
-        <v>8</v>
+      <c r="A22" s="2">
+        <v>4</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3">
+        <v>4</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>4</v>
-      </c>
-      <c r="B23">
-        <v>4</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>4</v>
-      </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>4</v>
-      </c>
-      <c r="B24">
-        <v>4</v>
-      </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24">
-        <v>6</v>
-      </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>4</v>
-      </c>
-      <c r="B25">
-        <v>4</v>
-      </c>
-      <c r="C25">
-        <v>3</v>
-      </c>
-      <c r="D25">
-        <v>8</v>
-      </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>4</v>
-      </c>
-      <c r="B26">
-        <v>5</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26">
-        <v>4</v>
-      </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>4</v>
-      </c>
-      <c r="B27">
-        <v>5</v>
-      </c>
-      <c r="C27">
-        <v>1</v>
-      </c>
-      <c r="D27">
-        <v>6</v>
-      </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>4</v>
-      </c>
-      <c r="B28">
-        <v>5</v>
-      </c>
-      <c r="C28">
-        <v>3</v>
-      </c>
-      <c r="D28">
-        <v>8</v>
-      </c>
       <c r="G28" s="1"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>